<commit_message>
Apply September Claude Pro receipt to Otani's draft invoice
Charge on 9/6 at 156.59499978 (from Anthropic's receipt): 20 USD base
= 3,132 yen, with the conversion noted in 備考.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GmiXe9RCHpFsdrbpadPUq2
</commit_message>
<xml_diff>
--- a/invoice_agent/otani_202609.xlsx
+++ b/invoice_agent/otani_202609.xlsx
@@ -500,6 +500,11 @@
       <c r="H2" s="1" t="n">
         <v>46295</v>
       </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Claude Pro代金20USDを9月6日付の日本銀行為替レート156.59499978にて円転換（消費税10%は他の項目とあわせて別途加算）</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -508,7 +513,7 @@
         </is>
       </c>
       <c r="B3" s="1" t="n">
-        <v>46295</v>
+        <v>46271</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -519,7 +524,7 @@
         <v>1</v>
       </c>
       <c r="E3" t="n">
-        <v>3153</v>
+        <v>3132</v>
       </c>
       <c r="F3" t="n">
         <v>10</v>

</xml_diff>